<commit_message>
Update accident report logic and associated test documentation
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/attached_assets/DEMO-PRUEBA_prueba_funcional_informe_siniestros_2026-10-09.xlsx
+++ b/attached_assets/DEMO-PRUEBA_prueba_funcional_informe_siniestros_2026-10-09.xlsx
@@ -34,28 +34,38 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -64,13 +74,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -418,99 +430,99 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="2" t="str">
         <v>REGISTRO DE VEHÍCULOS SINIESTRADOS</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2" s="2" t="str">
         <v>Empresa: DEMO-PRUEBA · NIT: 900000000-0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Generado: 11/10/2026, 4:59:23 a. m. · Período consultado: 09/10/2026 al 09/10/2026</v>
+      <c r="A3" s="2" t="str">
+        <v>Generado: 11/10/2026, 5:36:49 a. m. · Período consultado: 09/10/2026 al 09/10/2026</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5" s="2" t="str">
         <v>Fecha del siniestro</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B5" s="2" t="str">
         <v>Nivel de pérdida</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5" s="2" t="str">
         <v>Fatalidad (personas)</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5" s="2" t="str">
         <v>Heridos graves (personas)</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E5" s="2" t="str">
         <v>Heridos leves (personas)</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F5" s="2" t="str">
         <v>Choque simple (personas implicadas)</v>
       </c>
-      <c r="G5" t="str">
+      <c r="G5" s="2" t="str">
         <v>Placa del vehículo de la empresa</v>
       </c>
-      <c r="H5" t="str">
+      <c r="H5" s="2" t="str">
         <v>Nombre del conductor de la empresa</v>
       </c>
-      <c r="I5" t="str">
+      <c r="I5" s="2" t="str">
         <v>Identificación del conductor de la empresa</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J5" s="2" t="str">
         <v>Consecutivo del IPAT en RNAT/RUNT</v>
       </c>
-      <c r="K5" t="str">
+      <c r="K5" s="2" t="str">
         <v>Organismo de tránsito o autoridad que elaboró el IPAT</v>
       </c>
-      <c r="L5" t="str">
+      <c r="L5" s="2" t="str">
         <v>Número del acta del comité</v>
       </c>
-      <c r="M5" t="str">
+      <c r="M5" s="2" t="str">
         <v>Fecha del comité donde fue analizado</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6" s="2" t="str">
         <v>09/10/2026</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B6" s="2" t="str">
         <v>Choque simple: 2</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="2">
         <v>0</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>2</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G6" s="2" t="str">
         <v>TST001</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H6" s="2" t="str">
         <v>CONDUCTOR DE PRUEBA - NO REAL</v>
       </c>
-      <c r="I6" t="str">
+      <c r="I6" s="2" t="str">
         <v>PRUEBA-PESV-DAD9AD3288</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J6" s="2" t="str">
         <v>PRUEBA-IPAT-NO-REAL-PESV-DEMO-001</v>
       </c>
-      <c r="K6" t="str">
+      <c r="K6" s="2" t="str">
         <v>Autoridad de tránsito de prueba - NO REAL</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="2">
         <v>3</v>
       </c>
-      <c r="M6" t="str">
+      <c r="M6" s="2" t="str">
         <v>09/10/2026</v>
       </c>
     </row>

</xml_diff>